<commit_message>
refactor: replace single form submission timestamp with ISO and display formatted versions across all demo forms
</commit_message>
<xml_diff>
--- a/config/demo/forms/app/basic_health_checkup.xlsx
+++ b/config/demo/forms/app/basic_health_checkup.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="5" min="1" max="1"/>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="B93" s="12" t="inlineStr">
         <is>
-          <t>form_submit_timestamp</t>
+          <t>form_submit_timestamp_iso</t>
         </is>
       </c>
       <c r="C93" s="12" t="n"/>
@@ -2754,7 +2754,7 @@
       <c r="E93" s="12" t="n"/>
       <c r="F93" s="12" t="inlineStr">
         <is>
-          <t>if(${rapid_glucose} != '', now(), '')</t>
+          <t>if(${rapid_glucose} != '', format-date-time(now(), '%Y-%m-%dT%H:%M:%S+05:30'), '')</t>
         </is>
       </c>
       <c r="G93" s="12" t="n"/>
@@ -2762,23 +2762,40 @@
       <c r="I93" s="12" t="n"/>
     </row>
     <row r="94" ht="16" customHeight="1" s="6">
-      <c r="A94" s="11" t="inlineStr">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>form_submit_timestamp_display</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>if(${rapid_glucose} != '', format-date-time(now(), '%e-%b-%Y %H:%M:%S'), '')</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="11" t="inlineStr">
         <is>
           <t>end group</t>
         </is>
       </c>
-      <c r="B94" s="11" t="inlineStr">
+      <c r="B95" s="11" t="inlineStr">
         <is>
           <t>group_summary</t>
         </is>
       </c>
-      <c r="C94" s="11" t="n"/>
-      <c r="D94" s="11" t="n"/>
-      <c r="E94" s="11" t="n"/>
-      <c r="F94" s="11" t="n"/>
-      <c r="G94" s="11" t="n"/>
-      <c r="H94" s="11" t="n"/>
-      <c r="I94" s="11" t="n"/>
+      <c r="C95" s="11" t="n"/>
+      <c r="D95" s="11" t="n"/>
+      <c r="E95" s="11" t="n"/>
+      <c r="F95" s="11" t="n"/>
+      <c r="G95" s="11" t="n"/>
+      <c r="H95" s="11" t="n"/>
+      <c r="I95" s="11" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>